<commit_message>
Seed tennis pipeline regression test
</commit_message>
<xml_diff>
--- a/LSC_Tennis_Update_System.xlsx
+++ b/LSC_Tennis_Update_System.xlsx
@@ -851,7 +851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N500"/>
+  <dimension ref="A1:N503"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2750,6 +2750,186 @@
     </row>
     <row r="500">
       <c r="A500" s="9" t="n"/>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Men's Singles</t>
+        </is>
+      </c>
+      <c r="B501" s="10" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Test Opponent A</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Pipeline Test Event</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>Holder win</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>6–4 6–4</t>
+        </is>
+      </c>
+      <c r="K501" t="inlineStr">
+        <is>
+          <t>https://example.com/test-defence-1</t>
+        </is>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>PIPELINE TEST: holder defence</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Men's Singles</t>
+        </is>
+      </c>
+      <c r="B502" s="10" t="n">
+        <v>46285</v>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Test Challenger</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Pipeline Test Event</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>Challenger win</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>4–6 6–3 6–2</t>
+        </is>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>https://example.com/test-transfer</t>
+        </is>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>PIPELINE TEST: title transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Men's Singles</t>
+        </is>
+      </c>
+      <c r="B503" s="10" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Test Opponent B</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Pipeline Test Event</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>Holder win</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>7–5 6–3</t>
+        </is>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t>https://example.com/test-defence-2</t>
+        </is>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>PIPELINE TEST: new holder defence</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="6">

</xml_diff>

<commit_message>
Seed tennis pipeline test v2
</commit_message>
<xml_diff>
--- a/LSC_Tennis_Update_System.xlsx
+++ b/LSC_Tennis_Update_System.xlsx
@@ -496,7 +496,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -511,7 +510,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -526,8 +524,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
@@ -874,7 +870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N500"/>
+  <dimension ref="A1:N503"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2773,6 +2769,186 @@
     </row>
     <row r="500">
       <c r="A500" s="9" t="n"/>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Men's Singles</t>
+        </is>
+      </c>
+      <c r="B501" s="10" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Test Opponent A</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Pipeline Test Event</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>QF</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>Holder win</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>6–4 6–4</t>
+        </is>
+      </c>
+      <c r="K501" t="inlineStr">
+        <is>
+          <t>https://example.com/test-defence-1</t>
+        </is>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>PIPELINE TEST holder defence</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Men's Singles</t>
+        </is>
+      </c>
+      <c r="B502" s="10" t="n">
+        <v>46285</v>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Test Challenger</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Pipeline Test Event</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>Challenger win</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>4–6 6–3 6–2</t>
+        </is>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>https://example.com/test-transfer</t>
+        </is>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>PIPELINE TEST title transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Men's Singles</t>
+        </is>
+      </c>
+      <c r="B503" s="10" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Test Opponent B</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Pipeline Test Event</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>Holder win</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>7–5 6–3</t>
+        </is>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t>https://example.com/test-defence-2</t>
+        </is>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>PIPELINE TEST new holder defence</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="6">
@@ -2805,7 +2981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2858,7 +3034,6 @@
           <t>ITA</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Current men's baseline holder.</t>
@@ -2881,10 +3056,32 @@
           <t>KAZ</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Current women's baseline holder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Test Challenger</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PIPELINE TEST synthetic player</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Initialize generated tennis update data
</commit_message>
<xml_diff>
--- a/LSC_Tennis_Update_System.xlsx
+++ b/LSC_Tennis_Update_System.xlsx
@@ -11,9 +11,10 @@
     <sheet name="Baseline" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Updates" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Players" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Countries" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Lists" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Examples" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Aliases" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Countries" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Lists" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Examples" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -515,14 +516,14 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Player representation / flags</t>
+          <t>Player identity / representation</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Players contains one row per player. Choose a Country from the Countries lookup. The builder derives the Unicode flag automatically. Use Flag Override only for historical/special representations where a modern flag would be misleading.</t>
+          <t>For a new player, enter Player + Country. Leave Country Code and Player ID blank: the workflow fills them automatically. Approved historical name variants are resolved through the Aliases sheet. Use Flag Override only when needed.</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2813,6 +2814,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2841,6 +2843,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Player ID (auto)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2863,6 +2870,11 @@
           <t>Current men's baseline holder.</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>TP-018EED98ADD2</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2883,6 +2895,11 @@
       <c r="E3" t="inlineStr">
         <is>
           <t>Current women's baseline holder.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TP-1141A97BAAB9</t>
         </is>
       </c>
     </row>
@@ -2902,6 +2919,1555 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C90"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Alias</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Canonical Player</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Lineage scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alex Corretja</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Àlex Corretja</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Alex De Minaur</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Alex de Minaur</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Anders Jarryd</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Anders Järryd</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Andrés Gómez</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Balazs Taroczy</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Balázs Taróczy</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Barry Phillips Moore</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Barry Phillips-Moore</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bjorn Borg</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Björn Borg</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Carl Uwe Steeb</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Carl-Uwe Steeb</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Carlos Moya</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Carlos Moyá</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cedric Pioline</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cédric Pioline</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Diego Perez</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Diego Pérez</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Emilio Sanchez</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Emilio Sánchez</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Felix Auger Aliassime</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Felix Auger-Aliassime</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>German Lopez</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Germán López</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Goran Ivanisevic</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Goran Ivanišević</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Goran Prpic</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Goran Prpić</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Guillermo Garcia Lopez</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Guillermo Garcia-Lopez</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Guillermo Perez Roldan</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Guillermo Pérez-Roldán</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Heinz Gunthardt</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Heinz Günthardt</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Horacio De La Pena</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Horacio de la Peña</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ilie Nastase</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Ilie Năstase</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ivan Molina</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Iván Molina</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Jan Kodes</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Jan Kodeš</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Jan Lennard Struff</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Jan-Lennard Struff</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Javier Sanchez</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Javier Sánchez</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Jiri Hrebec</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Jiří Hřebec</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Joakim Nystrom</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Joakim Nyström</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>John Van Lottum</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>John van Lottum</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Jose Higueras</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>José Higueras</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Jose Luis Clerc</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>José Luis Clerc</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Karel Novacek</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Karel Nováček</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Karol Kucera</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Karol Kučera</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Malivai Washington</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MaliVai Washington</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Marc Kevin Goellner</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Marc-Kevin Goellner</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Marcello Lara</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Marcelo Lara</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Marcelo Rios</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Marcelo Ríos</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Martin Damm</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Martin Damm Sr</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Miloslav Mecir</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Miloslav Mečíř</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Nicolas Escude</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Nicolas Escudé</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Nikola Pilic</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nikola Pilić</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Patrik Kuhnen</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Patrik Kühnen</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Paul Henri Mathieu</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Paul-Henri Mathieu</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Paul Mcnamee</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Paul McNamee</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Peter Mcnamara</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Peter McNamara</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Raul Ramirez</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Raúl Ramírez</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Robert Vant Hof</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Robert Van't Hof</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Slobodan Zivojinovic</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Slobodan Živojinović</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Tomas Smid</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Tomáš Šmíd</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Vladimir Zednik</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Vladimir Zedník</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>MEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Agnes Szavay</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Ágnes Szávay</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Anna Schmiedlová</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Anna Karolína Schmiedlová</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Anne Gaelle Sidot</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Anne-Gaëlle Sidot</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Anne-Gaelle Sidot</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Anne-Gaëlle Sidot</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Arantxa Sanchez Vicario</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Arantxa Sánchez Vicario</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Asa Carlsson</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Åsa Svensson</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Betty Stove</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Betty Stöve</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Brenda Schultz McCarthy</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Brenda Schultz-McCarthy</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Conchita Martinez</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Conchita Martínez</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Daniela Hantuchova</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Daniela Hantuchová</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Francoise Durr</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Françoise Dürr</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Gigi Fernandez</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Gigi Fernández</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Hana Mandlikova</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Hana Mandlíková</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Helena Sukova</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Helena Suková</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Irina Spirlea</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Irina Spîrlea</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Jana Novotna</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Jana Novotná</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Jelena Dokic</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Jelena Dokić</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Jelena Kostanić</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Jelena Kostanić Tošić</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Joanne Russell</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>JoAnne Russell</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Julie Halard</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Julie Halard-Decugis</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Julie Halard Decugis</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Julie Halard-Decugis</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Karolina Sprem</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Karolina Šprem</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Katarina Studenikova</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Katarina Studeníková</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Kimberly Po Messerli</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Kimberly Po-Messerli</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Kimiko Date Krumm</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Kimiko Date-Krumm</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Kveta Peschke</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Květa Peschke</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Magdalena Rybarikova</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Magdaléna Rybáriková</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Magdalena Rybáriková</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Magdaléna Rybáriková</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Manuela Maleeva Fragniere</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Manuela Maleeva-Fragnière</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Manuela Maleeva-Fragniere</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Manuela Maleeva-Fragnière</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Mary Joe Fernandez</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Mary Joe Fernández</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Mima Jausovec</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Mima Jaušovec</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Mirjana Lučić</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Mirjana Lučić-Baroni</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Patricia Hy Boulais</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Patricia Hy-Boulais</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Petra Martic</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Petra Martić</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Regina Marsikova</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Regina Maršíková</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Ruxandra Dragomir</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Ruxandra Dragomir-Ilie</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Shahar Peer</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Shahar Pe'er</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Viktoria Kutuzova</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Viktoriya Kutuzova</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Åsa Carlsson/Svensson</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Åsa Svensson</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8416,7 +9982,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8605,7 +10171,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>